<commit_message>
docs(roadmap): update Excel roadmap and ROADMAP.md with minor corrections
- Owner: all phases now show "Product / Engineering" (was TIA/BP)
- Adapundi + OCBC redirect (E12 Phase 1) moved to Q1/end-of-March — it
  is a URL redirect, not API integration; already live in prototype
- Add backoffice note: separate backoffice app also targets Adapundi +
  OCBC by end of March 2026
- Add partner willingness dependency on E5, E6, E8, E10 — partner MOU
  required for partner-facing portal to be meaningful
- E7 (Scoring Engine) status: In Progress (was Todo/Start Here Next)
- Excel Gantt: E12 Ph.1 bar ends March W4; new orange band for partner
  MOU epics; E12 Ph.2 remains Jun; legend updated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OMM-2026-Roadmap.xlsx
+++ b/docs/OMM-2026-Roadmap.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,12 @@
       <name val="Arial"/>
       <color rgb="00111111"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -85,7 +91,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -129,6 +135,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF7ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0015803D"/>
       </patternFill>
     </fill>
@@ -149,11 +165,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
@@ -169,7 +180,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D97706"/>
+        <fgColor rgb="00F97316"/>
       </patternFill>
     </fill>
     <fill>
@@ -177,8 +188,13 @@
         <fgColor rgb="0094A3B8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D97706"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -258,11 +274,55 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -296,34 +356,18 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -335,7 +379,7 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -347,7 +391,19 @@
     <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -359,59 +415,83 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -779,17 +859,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -891,7 +971,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>Product / Engineering</t>
         </is>
       </c>
     </row>
@@ -903,12 +983,12 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Complete Merchant UX</t>
+          <t>Complete Merchant UX + Partner Redirect Cards</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>7 merchant pages, Scoring Engine, full Simulation flow</t>
+          <t>7 merchant pages, Scoring Engine, Simulation flow, Adapundi redirect, OCBC card</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -928,7 +1008,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>Product / Engineering</t>
         </is>
       </c>
     </row>
@@ -965,7 +1045,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>Product / Engineering</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1082,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>Product / Engineering</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1119,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>TIA</t>
+          <t>Product / Engineering</t>
         </is>
       </c>
     </row>
@@ -1076,648 +1156,738 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>BP</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="10" customHeight="1"/>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+          <t>Product / Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>⚠️  Note — Backoffice version: A separate backoffice application (not this web app) also targets Adapundi + OCBC integration by end of March 2026.</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="15" t="n"/>
+    </row>
+    <row r="12" ht="6" customHeight="1"/>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>⚠️  Partner dependency (E5, E6, E8, E10): Requires at least one partner to formally commit (signed MOU or equivalent). Without partner willingness, partner-facing portal and SLA mechanics cannot be meaningfully tested or operated end-to-end.</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="15" t="n"/>
+    </row>
+    <row r="14" ht="6" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Epic ID</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Epic Name</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Q1 2026</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="3" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Project Foundation &amp; Dev Environment</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Phase 1 — Foundation</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>28 Feb</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>None (Foundation Epic)</t>
         </is>
       </c>
-      <c r="H14" s="16" t="inlineStr">
+      <c r="H17" s="20" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>Design System &amp; Shared Components</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Phase 1 — Foundation</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>1 Mar</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>E1 (Boilerplate Setup)</t>
         </is>
       </c>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>Authentication &amp; RBAC</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D19" s="23" t="inlineStr">
         <is>
           <t>Phase 1 — Foundation</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>10 Mar</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G19" s="25" t="inlineStr">
         <is>
           <t>E2 (Design System)</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Scoring &amp; Matching Engine</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D20" s="23" t="inlineStr">
         <is>
           <t>Phase 2 — Merchant Flow</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>20 Mar</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="G17" s="25" t="inlineStr">
+      <c r="G20" s="25" t="inlineStr">
         <is>
           <t>E1 (DB Schema)</t>
         </is>
       </c>
-      <c r="H17" s="24" t="inlineStr">
-        <is>
-          <t>Todo — Start Here Next</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="H20" s="24" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>E4</t>
         </is>
       </c>
-      <c r="B18" s="19" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>Merchant Flow — Simulation &amp; Application</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="D21" s="23" t="inlineStr">
         <is>
           <t>Phase 2 — Merchant Flow</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>31 Mar</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="G21" s="25" t="inlineStr">
         <is>
           <t>E3 (Auth), E7 (Scoring)</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H21" s="24" t="inlineStr">
         <is>
           <t>In Progress (Frontend ✅ · API ⬜)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>E12
+(Phase 1)</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Partner Redirect — Adapundi + OCBC</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>Phase 2 — Merchant Flow</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>31 Mar</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>E4 (Merchant Flow) — URL redirect only, no API</t>
+        </is>
+      </c>
+      <c r="H22" s="24" t="inlineStr">
+        <is>
+          <t>Prototype ✅ · Production ⬜</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>E12 Phase 1: Adapundi redirect + OCBC 'Coming Soon' card — already live in prototype. Production deployment targets end of March. No API integration required.</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="15" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Q2 2026</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>SLA Management</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>Q1–Q2</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D25" s="23" t="inlineStr">
         <is>
           <t>Phase 3 — Partner Portal</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="E25" s="24" t="inlineStr">
         <is>
           <t>15 Apr</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr">
-        <is>
-          <t>E4 (Merchant Submit)</t>
-        </is>
-      </c>
-      <c r="H20" s="20" t="inlineStr">
+      <c r="G25" s="25" t="inlineStr">
+        <is>
+          <t>E4 (Merchant Submit) + Partner signed MOU ⚠️</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
         <is>
           <t>In Progress (Frontend ✅ · API ⬜)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>Partner Portal — Review &amp; Decision</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C26" s="28" t="inlineStr">
         <is>
           <t>Q1–Q2</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D26" s="27" t="inlineStr">
         <is>
           <t>Phase 3 — Partner Portal</t>
         </is>
       </c>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="E26" s="28" t="inlineStr">
         <is>
           <t>15 Apr</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G21" s="21" t="inlineStr">
-        <is>
-          <t>E4 (Merchant Flow), E7 (Score)</t>
-        </is>
-      </c>
-      <c r="H21" s="20" t="inlineStr">
-        <is>
-          <t>In Progress (Frontend ✅ · API ⬜)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="G26" s="29" t="inlineStr">
+        <is>
+          <t>E4 (Merchant Flow), E7 (Score) + Partner willingness / signed MOU ⚠️</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>Admin Portal — Operations &amp; Monitoring</t>
         </is>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C27" s="28" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D27" s="27" t="inlineStr">
         <is>
           <t>Phase 4 — Admin &amp; Data</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="E27" s="28" t="inlineStr">
         <is>
           <t>30 Apr</t>
         </is>
       </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G22" s="21" t="inlineStr">
-        <is>
-          <t>E5 (Partner), E8 (SLA)</t>
-        </is>
-      </c>
-      <c r="H22" s="20" t="inlineStr">
-        <is>
-          <t>In Progress (Frontend ✅ · API ⬜)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="G27" s="29" t="inlineStr">
+        <is>
+          <t>E5 (Partner), E8 (SLA) + Partner willingness / signed MOU ⚠️</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>E10</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>Data Team &amp; Management Views</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C28" s="28" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="D28" s="27" t="inlineStr">
         <is>
           <t>Phase 4 — Admin &amp; Data</t>
         </is>
       </c>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="E28" s="28" t="inlineStr">
         <is>
           <t>30 Apr</t>
         </is>
       </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>P1 - High</t>
         </is>
       </c>
-      <c r="G23" s="21" t="inlineStr">
-        <is>
-          <t>E4 (Merchant), E5 (Partner)</t>
-        </is>
-      </c>
-      <c r="H23" s="20" t="inlineStr">
-        <is>
-          <t>In Progress (Frontend ✅ · API ⬜)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>E4 (Merchant), E5 (Partner) + Partner data flowing ⚠️</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>E9</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>Database &amp; Seed Data</t>
         </is>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>Phase 5 — Backend APIs</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>31 May</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="G29" s="25" t="inlineStr">
         <is>
           <t>E1 (Migration runner)</t>
         </is>
       </c>
-      <c r="H24" s="20" t="inlineStr">
+      <c r="H29" s="24" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="22" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>E11</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B30" s="31" t="inlineStr">
         <is>
           <t>Testing &amp; QA</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C30" s="32" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D30" s="31" t="inlineStr">
         <is>
           <t>Phase 5 — Backend APIs</t>
         </is>
       </c>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="E30" s="32" t="inlineStr">
         <is>
           <t>31 May</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>P1 - High</t>
         </is>
       </c>
-      <c r="G25" s="25" t="inlineStr">
+      <c r="G30" s="33" t="inlineStr">
         <is>
           <t>All Epics</t>
         </is>
       </c>
-      <c r="H25" s="24" t="inlineStr">
+      <c r="H30" s="32" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Q2 – Q3 2026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="3" t="n"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="26" t="inlineStr">
-        <is>
-          <t>E12</t>
-        </is>
-      </c>
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t>Partner API Integration (Real)</t>
-        </is>
-      </c>
-      <c r="C27" s="28" t="inlineStr">
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="3" t="n"/>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="34" t="inlineStr">
+        <is>
+          <t>E12
+(Phase 2)</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>Partner API Integration (Full — Adapundi + OCBC)</t>
+        </is>
+      </c>
+      <c r="C32" s="36" t="inlineStr">
         <is>
           <t>Q2–Q3</t>
         </is>
       </c>
-      <c r="D27" s="27" t="inlineStr">
+      <c r="D32" s="35" t="inlineStr">
         <is>
           <t>Phase 6 — Partner Integration</t>
         </is>
       </c>
-      <c r="E27" s="28" t="inlineStr">
+      <c r="E32" s="36" t="inlineStr">
         <is>
           <t>30 Jun</t>
         </is>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G27" s="29" t="inlineStr">
-        <is>
-          <t>E5 (Partner Portal), API docs from partners</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="inlineStr">
-        <is>
-          <t>Phase 1 Redirect ✅ · Phase 2 API ⬜</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="G32" s="37" t="inlineStr">
+        <is>
+          <t>E5 (Partner Portal) + API docs + sandbox from Adapundi + OCBC ⚠️</t>
+        </is>
+      </c>
+      <c r="H32" s="36" t="inlineStr">
+        <is>
+          <t>Blocked on API docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="34" t="inlineStr">
         <is>
           <t>E13</t>
         </is>
       </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B33" s="35" t="inlineStr">
         <is>
           <t>Production Infrastructure &amp; Security</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C33" s="36" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="D28" s="31" t="inlineStr">
+      <c r="D33" s="35" t="inlineStr">
         <is>
           <t>Phase 6 — Partner Integration</t>
         </is>
       </c>
-      <c r="E28" s="32" t="inlineStr">
+      <c r="E33" s="36" t="inlineStr">
         <is>
           <t>30 Jun</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="G28" s="33" t="inlineStr">
-        <is>
-          <t>E11 (Tests), E12 (APIs)</t>
-        </is>
-      </c>
-      <c r="H28" s="32" t="inlineStr">
+      <c r="G33" s="37" t="inlineStr">
+        <is>
+          <t>E11 (Tests), E12 Phase 2 (APIs)</t>
+        </is>
+      </c>
+      <c r="H33" s="36" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A26:H26"/>
+  <mergeCells count="8">
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1729,14 +1899,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="4.5" customWidth="1" min="7" max="7"/>
     <col width="4.5" customWidth="1" min="8" max="8"/>
@@ -1813,148 +1983,148 @@
       <c r="V2" s="3" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="34" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Epic ID</t>
         </is>
       </c>
-      <c r="B3" s="34" t="inlineStr">
+      <c r="B3" s="38" t="inlineStr">
         <is>
           <t>Epic Name</t>
         </is>
       </c>
-      <c r="C3" s="34" t="inlineStr">
+      <c r="C3" s="38" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="D3" s="34" t="inlineStr">
+      <c r="D3" s="38" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E3" s="34" t="inlineStr">
+      <c r="E3" s="38" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="34" t="inlineStr">
+      <c r="F3" s="38" t="inlineStr">
         <is>
           <t>Target Date</t>
         </is>
       </c>
-      <c r="G3" s="35" t="inlineStr">
+      <c r="G3" s="39" t="inlineStr">
         <is>
           <t>March</t>
         </is>
       </c>
-      <c r="K3" s="35" t="inlineStr">
+      <c r="K3" s="39" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
-      <c r="O3" s="35" t="inlineStr">
+      <c r="O3" s="39" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="S3" s="35" t="inlineStr">
+      <c r="S3" s="39" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="G4" s="36" t="inlineStr">
+      <c r="G4" s="40" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="H4" s="36" t="inlineStr">
+      <c r="H4" s="40" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="I4" s="36" t="inlineStr">
+      <c r="I4" s="40" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="J4" s="36" t="inlineStr">
+      <c r="J4" s="40" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="K4" s="36" t="inlineStr">
+      <c r="K4" s="40" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="L4" s="36" t="inlineStr">
+      <c r="L4" s="40" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="M4" s="36" t="inlineStr">
+      <c r="M4" s="40" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="N4" s="36" t="inlineStr">
+      <c r="N4" s="40" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="O4" s="36" t="inlineStr">
+      <c r="O4" s="40" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="P4" s="36" t="inlineStr">
+      <c r="P4" s="40" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="Q4" s="36" t="inlineStr">
+      <c r="Q4" s="40" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="R4" s="36" t="inlineStr">
+      <c r="R4" s="40" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="S4" s="36" t="inlineStr">
+      <c r="S4" s="40" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="T4" s="36" t="inlineStr">
+      <c r="T4" s="40" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="U4" s="36" t="inlineStr">
+      <c r="U4" s="40" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="V4" s="36" t="inlineStr">
+      <c r="V4" s="40" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="37" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>E1</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Project Foundation &amp; Dev Environment</t>
+          <t>Project Foundation &amp; Dev Env</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -1962,12 +2132,12 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
+      <c r="D5" s="42" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="E5" s="39" t="inlineStr">
+      <c r="E5" s="43" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1977,25 +2147,25 @@
           <t>28 Feb</t>
         </is>
       </c>
-      <c r="G5" s="40" t="n"/>
-      <c r="H5" s="40" t="n"/>
-      <c r="I5" s="41" t="n"/>
-      <c r="J5" s="41" t="n"/>
-      <c r="K5" s="41" t="n"/>
-      <c r="L5" s="41" t="n"/>
-      <c r="M5" s="41" t="n"/>
-      <c r="N5" s="41" t="n"/>
-      <c r="O5" s="41" t="n"/>
-      <c r="P5" s="41" t="n"/>
-      <c r="Q5" s="41" t="n"/>
-      <c r="R5" s="41" t="n"/>
-      <c r="S5" s="41" t="n"/>
-      <c r="T5" s="41" t="n"/>
-      <c r="U5" s="41" t="n"/>
-      <c r="V5" s="41" t="n"/>
+      <c r="G5" s="44" t="n"/>
+      <c r="H5" s="44" t="n"/>
+      <c r="I5" s="45" t="n"/>
+      <c r="J5" s="45" t="n"/>
+      <c r="K5" s="45" t="n"/>
+      <c r="L5" s="45" t="n"/>
+      <c r="M5" s="45" t="n"/>
+      <c r="N5" s="45" t="n"/>
+      <c r="O5" s="45" t="n"/>
+      <c r="P5" s="45" t="n"/>
+      <c r="Q5" s="45" t="n"/>
+      <c r="R5" s="45" t="n"/>
+      <c r="S5" s="45" t="n"/>
+      <c r="T5" s="45" t="n"/>
+      <c r="U5" s="45" t="n"/>
+      <c r="V5" s="45" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
@@ -2010,7 +2180,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D6" s="38" t="inlineStr">
+      <c r="D6" s="42" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2025,25 +2195,25 @@
           <t>1 Mar</t>
         </is>
       </c>
-      <c r="G6" s="40" t="n"/>
-      <c r="H6" s="40" t="n"/>
-      <c r="I6" s="44" t="n"/>
-      <c r="J6" s="44" t="n"/>
-      <c r="K6" s="44" t="n"/>
-      <c r="L6" s="44" t="n"/>
-      <c r="M6" s="44" t="n"/>
-      <c r="N6" s="44" t="n"/>
-      <c r="O6" s="44" t="n"/>
-      <c r="P6" s="44" t="n"/>
-      <c r="Q6" s="44" t="n"/>
-      <c r="R6" s="44" t="n"/>
-      <c r="S6" s="44" t="n"/>
-      <c r="T6" s="44" t="n"/>
-      <c r="U6" s="44" t="n"/>
-      <c r="V6" s="44" t="n"/>
+      <c r="G6" s="44" t="n"/>
+      <c r="H6" s="44" t="n"/>
+      <c r="I6" s="47" t="n"/>
+      <c r="J6" s="47" t="n"/>
+      <c r="K6" s="47" t="n"/>
+      <c r="L6" s="47" t="n"/>
+      <c r="M6" s="47" t="n"/>
+      <c r="N6" s="47" t="n"/>
+      <c r="O6" s="47" t="n"/>
+      <c r="P6" s="47" t="n"/>
+      <c r="Q6" s="47" t="n"/>
+      <c r="R6" s="47" t="n"/>
+      <c r="S6" s="47" t="n"/>
+      <c r="T6" s="47" t="n"/>
+      <c r="U6" s="47" t="n"/>
+      <c r="V6" s="47" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
@@ -2058,12 +2228,12 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="E7" s="39" t="inlineStr">
+      <c r="E7" s="48" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -2073,25 +2243,25 @@
           <t>10 Mar</t>
         </is>
       </c>
-      <c r="G7" s="45" t="n"/>
-      <c r="H7" s="45" t="n"/>
-      <c r="I7" s="45" t="n"/>
-      <c r="J7" s="41" t="n"/>
-      <c r="K7" s="41" t="n"/>
-      <c r="L7" s="41" t="n"/>
-      <c r="M7" s="41" t="n"/>
-      <c r="N7" s="41" t="n"/>
-      <c r="O7" s="41" t="n"/>
-      <c r="P7" s="41" t="n"/>
-      <c r="Q7" s="41" t="n"/>
-      <c r="R7" s="41" t="n"/>
-      <c r="S7" s="41" t="n"/>
-      <c r="T7" s="41" t="n"/>
-      <c r="U7" s="41" t="n"/>
-      <c r="V7" s="41" t="n"/>
+      <c r="G7" s="49" t="n"/>
+      <c r="H7" s="49" t="n"/>
+      <c r="I7" s="49" t="n"/>
+      <c r="J7" s="45" t="n"/>
+      <c r="K7" s="45" t="n"/>
+      <c r="L7" s="45" t="n"/>
+      <c r="M7" s="45" t="n"/>
+      <c r="N7" s="45" t="n"/>
+      <c r="O7" s="45" t="n"/>
+      <c r="P7" s="45" t="n"/>
+      <c r="Q7" s="45" t="n"/>
+      <c r="R7" s="45" t="n"/>
+      <c r="S7" s="45" t="n"/>
+      <c r="T7" s="45" t="n"/>
+      <c r="U7" s="45" t="n"/>
+      <c r="V7" s="45" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
@@ -2106,14 +2276,14 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
+      <c r="D8" s="42" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
-        <is>
-          <t>Todo — Start Here Next</t>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -2121,25 +2291,25 @@
           <t>20 Mar</t>
         </is>
       </c>
-      <c r="G8" s="44" t="n"/>
-      <c r="H8" s="46" t="n"/>
-      <c r="I8" s="46" t="n"/>
-      <c r="J8" s="46" t="n"/>
-      <c r="K8" s="44" t="n"/>
-      <c r="L8" s="44" t="n"/>
-      <c r="M8" s="44" t="n"/>
-      <c r="N8" s="44" t="n"/>
-      <c r="O8" s="44" t="n"/>
-      <c r="P8" s="44" t="n"/>
-      <c r="Q8" s="44" t="n"/>
-      <c r="R8" s="44" t="n"/>
-      <c r="S8" s="44" t="n"/>
-      <c r="T8" s="44" t="n"/>
-      <c r="U8" s="44" t="n"/>
-      <c r="V8" s="44" t="n"/>
+      <c r="G8" s="47" t="n"/>
+      <c r="H8" s="49" t="n"/>
+      <c r="I8" s="49" t="n"/>
+      <c r="J8" s="49" t="n"/>
+      <c r="K8" s="47" t="n"/>
+      <c r="L8" s="47" t="n"/>
+      <c r="M8" s="47" t="n"/>
+      <c r="N8" s="47" t="n"/>
+      <c r="O8" s="47" t="n"/>
+      <c r="P8" s="47" t="n"/>
+      <c r="Q8" s="47" t="n"/>
+      <c r="R8" s="47" t="n"/>
+      <c r="S8" s="47" t="n"/>
+      <c r="T8" s="47" t="n"/>
+      <c r="U8" s="47" t="n"/>
+      <c r="V8" s="47" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>E4</t>
         </is>
@@ -2154,12 +2324,12 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D9" s="38" t="inlineStr">
+      <c r="D9" s="42" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
       </c>
-      <c r="E9" s="39" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -2169,461 +2339,517 @@
           <t>31 Mar</t>
         </is>
       </c>
-      <c r="G9" s="45" t="n"/>
-      <c r="H9" s="45" t="n"/>
-      <c r="I9" s="45" t="n"/>
-      <c r="J9" s="45" t="n"/>
-      <c r="K9" s="41" t="n"/>
-      <c r="L9" s="41" t="n"/>
-      <c r="M9" s="41" t="n"/>
-      <c r="N9" s="41" t="n"/>
-      <c r="O9" s="41" t="n"/>
-      <c r="P9" s="41" t="n"/>
-      <c r="Q9" s="41" t="n"/>
-      <c r="R9" s="41" t="n"/>
-      <c r="S9" s="41" t="n"/>
-      <c r="T9" s="41" t="n"/>
-      <c r="U9" s="41" t="n"/>
-      <c r="V9" s="41" t="n"/>
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="49" t="n"/>
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="45" t="n"/>
+      <c r="L9" s="45" t="n"/>
+      <c r="M9" s="45" t="n"/>
+      <c r="N9" s="45" t="n"/>
+      <c r="O9" s="45" t="n"/>
+      <c r="P9" s="45" t="n"/>
+      <c r="Q9" s="45" t="n"/>
+      <c r="R9" s="45" t="n"/>
+      <c r="S9" s="45" t="n"/>
+      <c r="T9" s="45" t="n"/>
+      <c r="U9" s="45" t="n"/>
+      <c r="V9" s="45" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>E12 Ph.1</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Adapundi Redirect + OCBC Card (→ prod)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D10" s="50" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>Prototype ✅ · Production ⬜</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>31 Mar</t>
+        </is>
+      </c>
+      <c r="G10" s="47" t="n"/>
+      <c r="H10" s="47" t="n"/>
+      <c r="I10" s="49" t="n"/>
+      <c r="J10" s="49" t="n"/>
+      <c r="K10" s="47" t="n"/>
+      <c r="L10" s="47" t="n"/>
+      <c r="M10" s="47" t="n"/>
+      <c r="N10" s="47" t="n"/>
+      <c r="O10" s="47" t="n"/>
+      <c r="P10" s="47" t="n"/>
+      <c r="Q10" s="47" t="n"/>
+      <c r="R10" s="47" t="n"/>
+      <c r="S10" s="47" t="n"/>
+      <c r="T10" s="47" t="n"/>
+      <c r="U10" s="47" t="n"/>
+      <c r="V10" s="47" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>SLA Management</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>SLA Management  ⚠️ partner MOU</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Q1–Q2</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D11" s="50" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="E10" s="43" t="inlineStr">
+      <c r="E11" s="51" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>15 Apr</t>
+        </is>
+      </c>
+      <c r="G11" s="45" t="n"/>
+      <c r="H11" s="45" t="n"/>
+      <c r="I11" s="52" t="n"/>
+      <c r="J11" s="52" t="n"/>
+      <c r="K11" s="52" t="n"/>
+      <c r="L11" s="52" t="n"/>
+      <c r="M11" s="45" t="n"/>
+      <c r="N11" s="45" t="n"/>
+      <c r="O11" s="45" t="n"/>
+      <c r="P11" s="45" t="n"/>
+      <c r="Q11" s="45" t="n"/>
+      <c r="R11" s="45" t="n"/>
+      <c r="S11" s="45" t="n"/>
+      <c r="T11" s="45" t="n"/>
+      <c r="U11" s="45" t="n"/>
+      <c r="V11" s="45" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Partner Portal  ⚠️ partner MOU</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Q1–Q2</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>15 Apr</t>
+        </is>
+      </c>
+      <c r="G12" s="47" t="n"/>
+      <c r="H12" s="47" t="n"/>
+      <c r="I12" s="52" t="n"/>
+      <c r="J12" s="52" t="n"/>
+      <c r="K12" s="52" t="n"/>
+      <c r="L12" s="52" t="n"/>
+      <c r="M12" s="47" t="n"/>
+      <c r="N12" s="47" t="n"/>
+      <c r="O12" s="47" t="n"/>
+      <c r="P12" s="47" t="n"/>
+      <c r="Q12" s="47" t="n"/>
+      <c r="R12" s="47" t="n"/>
+      <c r="S12" s="47" t="n"/>
+      <c r="T12" s="47" t="n"/>
+      <c r="U12" s="47" t="n"/>
+      <c r="V12" s="47" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Admin Portal  ⚠️ partner MOU</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="E13" s="51" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>30 Apr</t>
+        </is>
+      </c>
+      <c r="G13" s="45" t="n"/>
+      <c r="H13" s="45" t="n"/>
+      <c r="I13" s="45" t="n"/>
+      <c r="J13" s="45" t="n"/>
+      <c r="K13" s="52" t="n"/>
+      <c r="L13" s="52" t="n"/>
+      <c r="M13" s="52" t="n"/>
+      <c r="N13" s="52" t="n"/>
+      <c r="O13" s="45" t="n"/>
+      <c r="P13" s="45" t="n"/>
+      <c r="Q13" s="45" t="n"/>
+      <c r="R13" s="45" t="n"/>
+      <c r="S13" s="45" t="n"/>
+      <c r="T13" s="45" t="n"/>
+      <c r="U13" s="45" t="n"/>
+      <c r="V13" s="45" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Data &amp; Mgmt Views  ⚠️ partner MOU</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D14" s="53" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="E14" s="51" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>30 Apr</t>
+        </is>
+      </c>
+      <c r="G14" s="47" t="n"/>
+      <c r="H14" s="47" t="n"/>
+      <c r="I14" s="47" t="n"/>
+      <c r="J14" s="47" t="n"/>
+      <c r="K14" s="52" t="n"/>
+      <c r="L14" s="52" t="n"/>
+      <c r="M14" s="52" t="n"/>
+      <c r="N14" s="52" t="n"/>
+      <c r="O14" s="47" t="n"/>
+      <c r="P14" s="47" t="n"/>
+      <c r="Q14" s="47" t="n"/>
+      <c r="R14" s="47" t="n"/>
+      <c r="S14" s="47" t="n"/>
+      <c r="T14" s="47" t="n"/>
+      <c r="U14" s="47" t="n"/>
+      <c r="V14" s="47" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Database &amp; Seed Data</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D15" s="50" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>15 Apr</t>
-        </is>
-      </c>
-      <c r="G10" s="44" t="n"/>
-      <c r="H10" s="44" t="n"/>
-      <c r="I10" s="45" t="n"/>
-      <c r="J10" s="45" t="n"/>
-      <c r="K10" s="45" t="n"/>
-      <c r="L10" s="45" t="n"/>
-      <c r="M10" s="44" t="n"/>
-      <c r="N10" s="44" t="n"/>
-      <c r="O10" s="44" t="n"/>
-      <c r="P10" s="44" t="n"/>
-      <c r="Q10" s="44" t="n"/>
-      <c r="R10" s="44" t="n"/>
-      <c r="S10" s="44" t="n"/>
-      <c r="T10" s="44" t="n"/>
-      <c r="U10" s="44" t="n"/>
-      <c r="V10" s="44" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>E5</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Partner Portal — Review &amp; Decision</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Q1–Q2</t>
-        </is>
-      </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>31 May</t>
+        </is>
+      </c>
+      <c r="G15" s="45" t="n"/>
+      <c r="H15" s="45" t="n"/>
+      <c r="I15" s="45" t="n"/>
+      <c r="J15" s="49" t="n"/>
+      <c r="K15" s="49" t="n"/>
+      <c r="L15" s="49" t="n"/>
+      <c r="M15" s="49" t="n"/>
+      <c r="N15" s="49" t="n"/>
+      <c r="O15" s="49" t="n"/>
+      <c r="P15" s="49" t="n"/>
+      <c r="Q15" s="49" t="n"/>
+      <c r="R15" s="49" t="n"/>
+      <c r="S15" s="45" t="n"/>
+      <c r="T15" s="45" t="n"/>
+      <c r="U15" s="45" t="n"/>
+      <c r="V15" s="45" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="46" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Testing &amp; QA</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D16" s="53" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="E16" s="54" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>31 May</t>
+        </is>
+      </c>
+      <c r="G16" s="47" t="n"/>
+      <c r="H16" s="47" t="n"/>
+      <c r="I16" s="47" t="n"/>
+      <c r="J16" s="47" t="n"/>
+      <c r="K16" s="47" t="n"/>
+      <c r="L16" s="47" t="n"/>
+      <c r="M16" s="47" t="n"/>
+      <c r="N16" s="47" t="n"/>
+      <c r="O16" s="55" t="n"/>
+      <c r="P16" s="55" t="n"/>
+      <c r="Q16" s="55" t="n"/>
+      <c r="R16" s="55" t="n"/>
+      <c r="S16" s="47" t="n"/>
+      <c r="T16" s="47" t="n"/>
+      <c r="U16" s="47" t="n"/>
+      <c r="V16" s="47" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>E12 Ph.2</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Partner Full API (Adapundi + OCBC)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Q2–Q3</t>
+        </is>
+      </c>
+      <c r="D17" s="50" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="E11" s="39" t="inlineStr">
+      <c r="E17" s="56" t="inlineStr">
+        <is>
+          <t>Blocked on API docs</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>30 Jun</t>
+        </is>
+      </c>
+      <c r="G17" s="45" t="n"/>
+      <c r="H17" s="45" t="n"/>
+      <c r="I17" s="45" t="n"/>
+      <c r="J17" s="45" t="n"/>
+      <c r="K17" s="45" t="n"/>
+      <c r="L17" s="45" t="n"/>
+      <c r="M17" s="45" t="n"/>
+      <c r="N17" s="45" t="n"/>
+      <c r="O17" s="57" t="n"/>
+      <c r="P17" s="57" t="n"/>
+      <c r="Q17" s="57" t="n"/>
+      <c r="R17" s="57" t="n"/>
+      <c r="S17" s="57" t="n"/>
+      <c r="T17" s="57" t="n"/>
+      <c r="U17" s="57" t="n"/>
+      <c r="V17" s="57" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="46" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Production Infrastructure &amp; Security</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D18" s="50" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="E18" s="56" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>30 Jun</t>
+        </is>
+      </c>
+      <c r="G18" s="47" t="n"/>
+      <c r="H18" s="47" t="n"/>
+      <c r="I18" s="47" t="n"/>
+      <c r="J18" s="47" t="n"/>
+      <c r="K18" s="47" t="n"/>
+      <c r="L18" s="47" t="n"/>
+      <c r="M18" s="47" t="n"/>
+      <c r="N18" s="47" t="n"/>
+      <c r="O18" s="47" t="n"/>
+      <c r="P18" s="47" t="n"/>
+      <c r="Q18" s="47" t="n"/>
+      <c r="R18" s="47" t="n"/>
+      <c r="S18" s="57" t="n"/>
+      <c r="T18" s="57" t="n"/>
+      <c r="U18" s="57" t="n"/>
+      <c r="V18" s="57" t="n"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="58" t="inlineStr">
+        <is>
+          <t>LEGEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="59" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" s="60" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>15 Apr</t>
-        </is>
-      </c>
-      <c r="G11" s="41" t="n"/>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="45" t="n"/>
-      <c r="J11" s="45" t="n"/>
-      <c r="K11" s="45" t="n"/>
-      <c r="L11" s="45" t="n"/>
-      <c r="M11" s="41" t="n"/>
-      <c r="N11" s="41" t="n"/>
-      <c r="O11" s="41" t="n"/>
-      <c r="P11" s="41" t="n"/>
-      <c r="Q11" s="41" t="n"/>
-      <c r="R11" s="41" t="n"/>
-      <c r="S11" s="41" t="n"/>
-      <c r="T11" s="41" t="n"/>
-      <c r="U11" s="41" t="n"/>
-      <c r="V11" s="41" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>E6</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Admin Portal — Operations &amp; Monitor</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="D12" s="47" t="inlineStr">
-        <is>
-          <t>P0 - Critical</t>
-        </is>
-      </c>
-      <c r="E12" s="43" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>30 Apr</t>
-        </is>
-      </c>
-      <c r="G12" s="44" t="n"/>
-      <c r="H12" s="44" t="n"/>
-      <c r="I12" s="44" t="n"/>
-      <c r="J12" s="44" t="n"/>
-      <c r="K12" s="45" t="n"/>
-      <c r="L12" s="45" t="n"/>
-      <c r="M12" s="45" t="n"/>
-      <c r="N12" s="45" t="n"/>
-      <c r="O12" s="44" t="n"/>
-      <c r="P12" s="44" t="n"/>
-      <c r="Q12" s="44" t="n"/>
-      <c r="R12" s="44" t="n"/>
-      <c r="S12" s="44" t="n"/>
-      <c r="T12" s="44" t="n"/>
-      <c r="U12" s="44" t="n"/>
-      <c r="V12" s="44" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
-        <is>
-          <t>E10</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Data Team &amp; Management Views</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="D13" s="48" t="inlineStr">
-        <is>
-          <t>P1 - High</t>
-        </is>
-      </c>
-      <c r="E13" s="39" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>30 Apr</t>
-        </is>
-      </c>
-      <c r="G13" s="41" t="n"/>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="41" t="n"/>
-      <c r="K13" s="45" t="n"/>
-      <c r="L13" s="45" t="n"/>
-      <c r="M13" s="45" t="n"/>
-      <c r="N13" s="45" t="n"/>
-      <c r="O13" s="41" t="n"/>
-      <c r="P13" s="41" t="n"/>
-      <c r="Q13" s="41" t="n"/>
-      <c r="R13" s="41" t="n"/>
-      <c r="S13" s="41" t="n"/>
-      <c r="T13" s="41" t="n"/>
-      <c r="U13" s="41" t="n"/>
-      <c r="V13" s="41" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>E9</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Database &amp; Seed Data</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="D14" s="47" t="inlineStr">
-        <is>
-          <t>P0 - Critical</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>31 May</t>
-        </is>
-      </c>
-      <c r="G14" s="44" t="n"/>
-      <c r="H14" s="44" t="n"/>
-      <c r="I14" s="44" t="n"/>
-      <c r="J14" s="45" t="n"/>
-      <c r="K14" s="45" t="n"/>
-      <c r="L14" s="45" t="n"/>
-      <c r="M14" s="45" t="n"/>
-      <c r="N14" s="45" t="n"/>
-      <c r="O14" s="45" t="n"/>
-      <c r="P14" s="45" t="n"/>
-      <c r="Q14" s="45" t="n"/>
-      <c r="R14" s="45" t="n"/>
-      <c r="S14" s="44" t="n"/>
-      <c r="T14" s="44" t="n"/>
-      <c r="U14" s="44" t="n"/>
-      <c r="V14" s="44" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t>E11</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Testing &amp; QA</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="D15" s="48" t="inlineStr">
-        <is>
-          <t>P1 - High</t>
-        </is>
-      </c>
-      <c r="E15" s="39" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>31 May</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="41" t="n"/>
-      <c r="K15" s="41" t="n"/>
-      <c r="L15" s="41" t="n"/>
-      <c r="M15" s="41" t="n"/>
-      <c r="N15" s="41" t="n"/>
-      <c r="O15" s="46" t="n"/>
-      <c r="P15" s="46" t="n"/>
-      <c r="Q15" s="46" t="n"/>
-      <c r="R15" s="46" t="n"/>
-      <c r="S15" s="41" t="n"/>
-      <c r="T15" s="41" t="n"/>
-      <c r="U15" s="41" t="n"/>
-      <c r="V15" s="41" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>E12</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Partner API Integration (Real)</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Q2–Q3</t>
-        </is>
-      </c>
-      <c r="D16" s="47" t="inlineStr">
-        <is>
-          <t>P0 - Critical</t>
-        </is>
-      </c>
-      <c r="E16" s="43" t="inlineStr">
-        <is>
-          <t>Phase 1 Redirect ✅ · Phase 2 API ⬜</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>30 Jun</t>
-        </is>
-      </c>
-      <c r="G16" s="44" t="n"/>
-      <c r="H16" s="44" t="n"/>
-      <c r="I16" s="44" t="n"/>
-      <c r="J16" s="44" t="n"/>
-      <c r="K16" s="44" t="n"/>
-      <c r="L16" s="44" t="n"/>
-      <c r="M16" s="44" t="n"/>
-      <c r="N16" s="44" t="n"/>
-      <c r="O16" s="49" t="n"/>
-      <c r="P16" s="49" t="n"/>
-      <c r="Q16" s="49" t="n"/>
-      <c r="R16" s="49" t="n"/>
-      <c r="S16" s="49" t="n"/>
-      <c r="T16" s="49" t="n"/>
-      <c r="U16" s="49" t="n"/>
-      <c r="V16" s="49" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>E13</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Production Infrastructure &amp; Security</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="D17" s="47" t="inlineStr">
-        <is>
-          <t>P0 - Critical</t>
-        </is>
-      </c>
-      <c r="E17" s="39" t="inlineStr">
-        <is>
-          <t>Phase 2</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>30 Jun</t>
-        </is>
-      </c>
-      <c r="G17" s="41" t="n"/>
-      <c r="H17" s="41" t="n"/>
-      <c r="I17" s="41" t="n"/>
-      <c r="J17" s="41" t="n"/>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="41" t="n"/>
-      <c r="M17" s="41" t="n"/>
-      <c r="N17" s="41" t="n"/>
-      <c r="O17" s="41" t="n"/>
-      <c r="P17" s="41" t="n"/>
-      <c r="Q17" s="41" t="n"/>
-      <c r="R17" s="41" t="n"/>
-      <c r="S17" s="50" t="n"/>
-      <c r="T17" s="50" t="n"/>
-      <c r="U17" s="50" t="n"/>
-      <c r="V17" s="50" t="n"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="51" t="inlineStr">
-        <is>
-          <t>LEGEND</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="52" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E21" s="53" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="I21" s="54" t="inlineStr">
+      <c r="K22" s="61" t="inlineStr">
         <is>
           <t>Todo / Planned</t>
         </is>
       </c>
-      <c r="M21" s="55" t="inlineStr">
-        <is>
-          <t>Phase 1 ✅ · Phase 2 ⬜</t>
-        </is>
-      </c>
-      <c r="Q21" s="56" t="inlineStr">
-        <is>
-          <t>Phase 2 Only</t>
+      <c r="P22" s="62" t="inlineStr">
+        <is>
+          <t>Phase 1 Redirect ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="63" t="inlineStr">
+        <is>
+          <t>⚠️ Needs Partner MOU</t>
+        </is>
+      </c>
+      <c r="F23" s="64" t="inlineStr">
+        <is>
+          <t>Blocked / Phase 2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A2:V2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="P22:T22"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="O3:R3"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="K22:O22"/>
     <mergeCell ref="S3:V3"/>
+    <mergeCell ref="F23:J23"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="G3:J3"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="A1:V1"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A3:A4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="O3:R3"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="I21:L21"/>
-    <mergeCell ref="M21:P21"/>
-    <mergeCell ref="Q21:T21"/>
-    <mergeCell ref="A20:V20"/>
+    <mergeCell ref="A21:V21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(roadmap): add Master Timeline Visual and Table sheets to Excel roadmap
Added two new sheets to OMM-2026-Roadmap.xlsx (now 4 sheets total):
- Sheet 3 "Master Timeline (Visual)": Phase boxes with arrows, module milestone
  grid with colored status bars, revenue linkage, and dependency sidebar
- Sheet 4 "Master Timeline (Table)": Executive summary + dependencies, module
  Gantt with month columns (Mar–Jul), revenue linkage table with status cells

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OMM-2026-Roadmap.xlsx
+++ b/docs/OMM-2026-Roadmap.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Product Roadmap" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Epic Timeline" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Master Timeline (Visual)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Master Timeline (Table)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +92,116 @@
       <color rgb="001E3A8A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F2D5E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002563EB"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00CBD5E1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00BFDBFE"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F2D5E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000F2D5E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00475569"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000F2D5E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F2D5E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F2D5E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00475569"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -193,8 +303,48 @@
         <fgColor rgb="00D97706"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F2D5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B1F4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E7490"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFDBFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000891B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0064748B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003B82F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -318,11 +468,162 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00EEEEEE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00EEEEEE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00EEEEEE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00EEEEEE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -494,6 +795,219 @@
     <xf numFmtId="0" fontId="9" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="21" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -902,37 +1416,37 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>Key Deliverables</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="38" t="inlineStr">
         <is>
           <t>Target Go Live</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="38" t="inlineStr">
         <is>
           <t>Revenue Impact</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="38" t="inlineStr">
         <is>
           <t>Risk Level</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="38" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
@@ -1191,42 +1705,42 @@
     </row>
     <row r="14" ht="6" customHeight="1"/>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>Epic ID</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="38" t="inlineStr">
         <is>
           <t>Epic Name</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="38" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="38" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="38" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="38" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2018,23 +2532,41 @@
           <t>March</t>
         </is>
       </c>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="3" t="n"/>
       <c r="K3" s="39" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="3" t="n"/>
       <c r="O3" s="39" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="3" t="n"/>
       <c r="S3" s="39" t="inlineStr">
         <is>
           <t>June</t>
         </is>
       </c>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="2" t="n"/>
+      <c r="V3" s="3" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="65" t="n"/>
+      <c r="B4" s="65" t="n"/>
+      <c r="C4" s="65" t="n"/>
+      <c r="D4" s="65" t="n"/>
+      <c r="E4" s="65" t="n"/>
+      <c r="F4" s="65" t="n"/>
       <c r="G4" s="40" t="inlineStr">
         <is>
           <t>W1</t>
@@ -2132,7 +2664,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="61" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2180,7 +2712,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D6" s="42" t="inlineStr">
+      <c r="D6" s="61" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2228,7 +2760,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="61" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2276,7 +2808,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
+      <c r="D8" s="61" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2324,7 +2856,7 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="61" t="inlineStr">
         <is>
           <t>P0 - Blocker</t>
         </is>
@@ -2801,21 +3333,37 @@
           <t>Done</t>
         </is>
       </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="3" t="n"/>
       <c r="F22" s="60" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="3" t="n"/>
       <c r="K22" s="61" t="inlineStr">
         <is>
           <t>Todo / Planned</t>
         </is>
       </c>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="3" t="n"/>
       <c r="P22" s="62" t="inlineStr">
         <is>
           <t>Phase 1 Redirect ✅</t>
         </is>
       </c>
+      <c r="Q22" s="2" t="n"/>
+      <c r="R22" s="2" t="n"/>
+      <c r="S22" s="2" t="n"/>
+      <c r="T22" s="3" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="63" t="inlineStr">
@@ -2823,11 +3371,19 @@
           <t>⚠️ Needs Partner MOU</t>
         </is>
       </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="3" t="n"/>
       <c r="F23" s="64" t="inlineStr">
         <is>
           <t>Blocked / Phase 2</t>
         </is>
       </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -2853,4 +3409,1698 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="4" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="18" max="18"/>
+    <col width="4" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="9" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>OLSERA MITRA MODAL — PROGRAM MASTER TIMELINE 2026</t>
+        </is>
+      </c>
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="67" t="n"/>
+      <c r="J1" s="67" t="n"/>
+      <c r="K1" s="67" t="n"/>
+      <c r="L1" s="67" t="n"/>
+      <c r="M1" s="67" t="n"/>
+      <c r="N1" s="67" t="n"/>
+      <c r="O1" s="67" t="n"/>
+      <c r="P1" s="67" t="n"/>
+      <c r="Q1" s="67" t="n"/>
+      <c r="R1" s="67" t="n"/>
+      <c r="S1" s="67" t="n"/>
+      <c r="T1" s="67" t="n"/>
+      <c r="U1" s="67" t="n"/>
+      <c r="V1" s="68" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="69" t="inlineStr">
+        <is>
+          <t>Financial Infrastructure Development &amp; Commercial Rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="70" t="inlineStr">
+        <is>
+          <t>EXECUTIVE PHASE OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="71" t="inlineStr">
+        <is>
+          <t>PHASE 1  FOUNDATION</t>
+        </is>
+      </c>
+      <c r="B5" s="67" t="n"/>
+      <c r="C5" s="67" t="n"/>
+      <c r="D5" s="67" t="n"/>
+      <c r="E5" s="67" t="n"/>
+      <c r="F5" s="68" t="n"/>
+      <c r="G5" s="72" t="inlineStr"/>
+      <c r="H5" s="73" t="inlineStr">
+        <is>
+          <t>PHASE 2  INTEGRATION</t>
+        </is>
+      </c>
+      <c r="I5" s="67" t="n"/>
+      <c r="J5" s="67" t="n"/>
+      <c r="K5" s="67" t="n"/>
+      <c r="L5" s="67" t="n"/>
+      <c r="M5" s="68" t="n"/>
+      <c r="N5" s="72" t="inlineStr"/>
+      <c r="O5" s="74" t="inlineStr">
+        <is>
+          <t>PHASE 3  COMMERCIALIZATION</t>
+        </is>
+      </c>
+      <c r="P5" s="67" t="n"/>
+      <c r="Q5" s="67" t="n"/>
+      <c r="R5" s="67" t="n"/>
+      <c r="S5" s="67" t="n"/>
+      <c r="T5" s="67" t="n"/>
+      <c r="U5" s="67" t="n"/>
+      <c r="V5" s="68" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="75" t="inlineStr">
+        <is>
+          <t>Mar – Apr 2026</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="n"/>
+      <c r="C6" s="67" t="n"/>
+      <c r="D6" s="67" t="n"/>
+      <c r="E6" s="67" t="n"/>
+      <c r="F6" s="68" t="n"/>
+      <c r="G6" s="72" t="inlineStr"/>
+      <c r="H6" s="76" t="inlineStr">
+        <is>
+          <t>Apr – May 2026</t>
+        </is>
+      </c>
+      <c r="I6" s="67" t="n"/>
+      <c r="J6" s="67" t="n"/>
+      <c r="K6" s="67" t="n"/>
+      <c r="L6" s="67" t="n"/>
+      <c r="M6" s="68" t="n"/>
+      <c r="N6" s="72" t="inlineStr"/>
+      <c r="O6" s="77" t="inlineStr">
+        <is>
+          <t>Jun – Jul 2026</t>
+        </is>
+      </c>
+      <c r="P6" s="67" t="n"/>
+      <c r="Q6" s="67" t="n"/>
+      <c r="R6" s="67" t="n"/>
+      <c r="S6" s="67" t="n"/>
+      <c r="T6" s="67" t="n"/>
+      <c r="U6" s="67" t="n"/>
+      <c r="V6" s="68" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="78" t="inlineStr">
+        <is>
+          <t>Core Platform Build</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="n"/>
+      <c r="C7" s="67" t="n"/>
+      <c r="D7" s="67" t="n"/>
+      <c r="E7" s="67" t="n"/>
+      <c r="F7" s="68" t="n"/>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="H7" s="79" t="inlineStr">
+        <is>
+          <t>Backend APIs &amp; Partner Portal</t>
+        </is>
+      </c>
+      <c r="I7" s="67" t="n"/>
+      <c r="J7" s="67" t="n"/>
+      <c r="K7" s="67" t="n"/>
+      <c r="L7" s="67" t="n"/>
+      <c r="M7" s="68" t="n"/>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>→</t>
+        </is>
+      </c>
+      <c r="O7" s="80" t="inlineStr">
+        <is>
+          <t>Merchant Rollout &amp; Monetization</t>
+        </is>
+      </c>
+      <c r="P7" s="67" t="n"/>
+      <c r="Q7" s="67" t="n"/>
+      <c r="R7" s="67" t="n"/>
+      <c r="S7" s="67" t="n"/>
+      <c r="T7" s="67" t="n"/>
+      <c r="U7" s="67" t="n"/>
+      <c r="V7" s="68" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="81" t="inlineStr">
+        <is>
+          <t>5-portal prototype • Auth • Scoring engine</t>
+        </is>
+      </c>
+      <c r="B8" s="67" t="n"/>
+      <c r="C8" s="67" t="n"/>
+      <c r="D8" s="67" t="n"/>
+      <c r="E8" s="67" t="n"/>
+      <c r="F8" s="68" t="n"/>
+      <c r="G8" s="72" t="inlineStr"/>
+      <c r="H8" s="82" t="inlineStr">
+        <is>
+          <t>All API endpoints live • Partner MOU required</t>
+        </is>
+      </c>
+      <c r="I8" s="67" t="n"/>
+      <c r="J8" s="67" t="n"/>
+      <c r="K8" s="67" t="n"/>
+      <c r="L8" s="67" t="n"/>
+      <c r="M8" s="68" t="n"/>
+      <c r="N8" s="72" t="inlineStr"/>
+      <c r="O8" s="83" t="inlineStr">
+        <is>
+          <t>1,000 merchants onboarded • Referral fee revenue</t>
+        </is>
+      </c>
+      <c r="P8" s="67" t="n"/>
+      <c r="Q8" s="67" t="n"/>
+      <c r="R8" s="67" t="n"/>
+      <c r="S8" s="67" t="n"/>
+      <c r="T8" s="67" t="n"/>
+      <c r="U8" s="67" t="n"/>
+      <c r="V8" s="68" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="84" t="inlineStr">
+        <is>
+          <t>Go-Live: Apr '26</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="n"/>
+      <c r="C9" s="67" t="n"/>
+      <c r="D9" s="67" t="n"/>
+      <c r="E9" s="67" t="n"/>
+      <c r="F9" s="68" t="n"/>
+      <c r="G9" s="72" t="inlineStr"/>
+      <c r="H9" s="85" t="inlineStr">
+        <is>
+          <t>Go-Live: May '26</t>
+        </is>
+      </c>
+      <c r="I9" s="67" t="n"/>
+      <c r="J9" s="67" t="n"/>
+      <c r="K9" s="67" t="n"/>
+      <c r="L9" s="67" t="n"/>
+      <c r="M9" s="68" t="n"/>
+      <c r="N9" s="72" t="inlineStr"/>
+      <c r="O9" s="86" t="inlineStr">
+        <is>
+          <t>Go-Live: Jul '26</t>
+        </is>
+      </c>
+      <c r="P9" s="67" t="n"/>
+      <c r="Q9" s="67" t="n"/>
+      <c r="R9" s="67" t="n"/>
+      <c r="S9" s="67" t="n"/>
+      <c r="T9" s="67" t="n"/>
+      <c r="U9" s="67" t="n"/>
+      <c r="V9" s="68" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="87" t="inlineStr">
+        <is>
+          <t>Risk: Low</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="n"/>
+      <c r="C10" s="67" t="n"/>
+      <c r="D10" s="67" t="n"/>
+      <c r="E10" s="67" t="n"/>
+      <c r="F10" s="68" t="n"/>
+      <c r="G10" s="72" t="inlineStr"/>
+      <c r="H10" s="88" t="inlineStr">
+        <is>
+          <t>Risk: Medium</t>
+        </is>
+      </c>
+      <c r="I10" s="67" t="n"/>
+      <c r="J10" s="67" t="n"/>
+      <c r="K10" s="67" t="n"/>
+      <c r="L10" s="67" t="n"/>
+      <c r="M10" s="68" t="n"/>
+      <c r="N10" s="72" t="inlineStr"/>
+      <c r="O10" s="89" t="inlineStr">
+        <is>
+          <t>Risk: High</t>
+        </is>
+      </c>
+      <c r="P10" s="67" t="n"/>
+      <c r="Q10" s="67" t="n"/>
+      <c r="R10" s="67" t="n"/>
+      <c r="S10" s="67" t="n"/>
+      <c r="T10" s="67" t="n"/>
+      <c r="U10" s="67" t="n"/>
+      <c r="V10" s="68" t="n"/>
+    </row>
+    <row r="11" ht="14" customHeight="1"/>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>MODULE MILESTONE BREAKDOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="90" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B13" s="68" t="n"/>
+      <c r="C13" s="91" t="inlineStr">
+        <is>
+          <t>Merchant Flow Engine</t>
+        </is>
+      </c>
+      <c r="D13" s="67" t="n"/>
+      <c r="E13" s="67" t="n"/>
+      <c r="F13" s="67" t="n"/>
+      <c r="G13" s="68" t="n"/>
+      <c r="H13" s="92" t="inlineStr">
+        <is>
+          <t>Scoring Engine</t>
+        </is>
+      </c>
+      <c r="I13" s="67" t="n"/>
+      <c r="J13" s="67" t="n"/>
+      <c r="K13" s="68" t="n"/>
+      <c r="L13" s="93" t="inlineStr">
+        <is>
+          <t>Partner Portal ⚠</t>
+        </is>
+      </c>
+      <c r="M13" s="67" t="n"/>
+      <c r="N13" s="67" t="n"/>
+      <c r="O13" s="68" t="n"/>
+      <c r="P13" s="94" t="inlineStr">
+        <is>
+          <t>Admin &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="Q13" s="67" t="n"/>
+      <c r="R13" s="67" t="n"/>
+      <c r="S13" s="68" t="n"/>
+      <c r="T13" s="90" t="inlineStr">
+        <is>
+          <t>DEPENDENCY MAP</t>
+        </is>
+      </c>
+      <c r="U13" s="67" t="n"/>
+      <c r="V13" s="68" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="95" t="inlineStr">
+        <is>
+          <t>Phase / Period</t>
+        </is>
+      </c>
+      <c r="B14" s="68" t="n"/>
+      <c r="C14" s="96" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="67" t="n"/>
+      <c r="G14" s="68" t="n"/>
+      <c r="H14" s="97" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I14" s="67" t="n"/>
+      <c r="J14" s="67" t="n"/>
+      <c r="K14" s="68" t="n"/>
+      <c r="L14" s="98" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="M14" s="67" t="n"/>
+      <c r="N14" s="67" t="n"/>
+      <c r="O14" s="68" t="n"/>
+      <c r="P14" s="99" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="Q14" s="67" t="n"/>
+      <c r="R14" s="67" t="n"/>
+      <c r="S14" s="68" t="n"/>
+      <c r="T14" s="95" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="U14" s="95" t="inlineStr">
+        <is>
+          <t>Risk Impact</t>
+        </is>
+      </c>
+      <c r="V14" s="95" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="100" t="inlineStr">
+        <is>
+          <t>Platform Design
+&amp; Prototyping
+(Mar – Apr)</t>
+        </is>
+      </c>
+      <c r="B15" s="101" t="n"/>
+      <c r="C15" s="91" t="inlineStr">
+        <is>
+          <t>✓ Done</t>
+        </is>
+      </c>
+      <c r="D15" s="67" t="n"/>
+      <c r="E15" s="67" t="n"/>
+      <c r="F15" s="67" t="n"/>
+      <c r="G15" s="68" t="n"/>
+      <c r="H15" s="92" t="inlineStr">
+        <is>
+          <t>✓ Done</t>
+        </is>
+      </c>
+      <c r="I15" s="67" t="n"/>
+      <c r="J15" s="67" t="n"/>
+      <c r="K15" s="68" t="n"/>
+      <c r="L15" s="93" t="inlineStr">
+        <is>
+          <t>✓ Done</t>
+        </is>
+      </c>
+      <c r="M15" s="67" t="n"/>
+      <c r="N15" s="67" t="n"/>
+      <c r="O15" s="68" t="n"/>
+      <c r="P15" s="94" t="inlineStr">
+        <is>
+          <t>✓ Done</t>
+        </is>
+      </c>
+      <c r="Q15" s="67" t="n"/>
+      <c r="R15" s="67" t="n"/>
+      <c r="S15" s="68" t="n"/>
+      <c r="T15" s="102" t="inlineStr">
+        <is>
+          <t>Partner API Access</t>
+        </is>
+      </c>
+      <c r="U15" s="103" t="inlineStr">
+        <is>
+          <t>High ⚠</t>
+        </is>
+      </c>
+      <c r="V15" s="104" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="8" customHeight="1">
+      <c r="A16" s="105" t="n"/>
+      <c r="B16" s="106" t="n"/>
+      <c r="C16" s="107" t="n"/>
+      <c r="D16" s="107" t="n"/>
+      <c r="E16" s="107" t="n"/>
+      <c r="F16" s="107" t="n"/>
+      <c r="G16" s="107" t="n"/>
+      <c r="H16" s="107" t="n"/>
+      <c r="I16" s="107" t="n"/>
+      <c r="J16" s="107" t="n"/>
+      <c r="K16" s="107" t="n"/>
+      <c r="L16" s="108" t="n"/>
+      <c r="M16" s="108" t="n"/>
+      <c r="N16" s="108" t="n"/>
+      <c r="O16" s="108" t="n"/>
+      <c r="P16" s="108" t="n"/>
+      <c r="Q16" s="108" t="n"/>
+      <c r="R16" s="108" t="n"/>
+      <c r="S16" s="108" t="n"/>
+      <c r="T16" s="109" t="inlineStr"/>
+      <c r="U16" s="109" t="inlineStr"/>
+      <c r="V16" s="109" t="inlineStr"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="100" t="inlineStr">
+        <is>
+          <t>Engine Dev
+&amp; API Build
+(Apr – May)</t>
+        </is>
+      </c>
+      <c r="B17" s="101" t="n"/>
+      <c r="C17" s="110" t="inlineStr">
+        <is>
+          <t>▶ Active</t>
+        </is>
+      </c>
+      <c r="D17" s="67" t="n"/>
+      <c r="E17" s="67" t="n"/>
+      <c r="F17" s="67" t="n"/>
+      <c r="G17" s="68" t="n"/>
+      <c r="H17" s="111" t="inlineStr">
+        <is>
+          <t>▶ Active</t>
+        </is>
+      </c>
+      <c r="I17" s="67" t="n"/>
+      <c r="J17" s="67" t="n"/>
+      <c r="K17" s="68" t="n"/>
+      <c r="L17" s="89" t="inlineStr">
+        <is>
+          <t>⚠ At Risk</t>
+        </is>
+      </c>
+      <c r="M17" s="67" t="n"/>
+      <c r="N17" s="67" t="n"/>
+      <c r="O17" s="68" t="n"/>
+      <c r="P17" s="87" t="inlineStr">
+        <is>
+          <t>▶ Active</t>
+        </is>
+      </c>
+      <c r="Q17" s="67" t="n"/>
+      <c r="R17" s="67" t="n"/>
+      <c r="S17" s="68" t="n"/>
+      <c r="T17" s="102" t="inlineStr">
+        <is>
+          <t>Data Schema Final.</t>
+        </is>
+      </c>
+      <c r="U17" s="112" t="inlineStr">
+        <is>
+          <t>Medium △</t>
+        </is>
+      </c>
+      <c r="V17" s="104" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="8" customHeight="1">
+      <c r="A18" s="105" t="n"/>
+      <c r="B18" s="106" t="n"/>
+      <c r="C18" s="107" t="n"/>
+      <c r="D18" s="107" t="n"/>
+      <c r="E18" s="107" t="n"/>
+      <c r="F18" s="107" t="n"/>
+      <c r="G18" s="107" t="n"/>
+      <c r="H18" s="107" t="n"/>
+      <c r="I18" s="107" t="n"/>
+      <c r="J18" s="107" t="n"/>
+      <c r="K18" s="107" t="n"/>
+      <c r="L18" s="108" t="n"/>
+      <c r="M18" s="108" t="n"/>
+      <c r="N18" s="108" t="n"/>
+      <c r="O18" s="108" t="n"/>
+      <c r="P18" s="108" t="n"/>
+      <c r="Q18" s="108" t="n"/>
+      <c r="R18" s="108" t="n"/>
+      <c r="S18" s="108" t="n"/>
+      <c r="T18" s="109" t="inlineStr"/>
+      <c r="U18" s="109" t="inlineStr"/>
+      <c r="V18" s="109" t="inlineStr"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="100" t="inlineStr">
+        <is>
+          <t>System Testing
+&amp; QA
+(May)</t>
+        </is>
+      </c>
+      <c r="B19" s="101" t="n"/>
+      <c r="C19" s="113" t="inlineStr">
+        <is>
+          <t>○ Planned</t>
+        </is>
+      </c>
+      <c r="D19" s="67" t="n"/>
+      <c r="E19" s="67" t="n"/>
+      <c r="F19" s="67" t="n"/>
+      <c r="G19" s="68" t="n"/>
+      <c r="H19" s="113" t="inlineStr">
+        <is>
+          <t>○ Planned</t>
+        </is>
+      </c>
+      <c r="I19" s="67" t="n"/>
+      <c r="J19" s="67" t="n"/>
+      <c r="K19" s="68" t="n"/>
+      <c r="L19" s="114" t="inlineStr">
+        <is>
+          <t>— Blocked</t>
+        </is>
+      </c>
+      <c r="M19" s="67" t="n"/>
+      <c r="N19" s="67" t="n"/>
+      <c r="O19" s="68" t="n"/>
+      <c r="P19" s="113" t="inlineStr">
+        <is>
+          <t>○ Planned</t>
+        </is>
+      </c>
+      <c r="Q19" s="67" t="n"/>
+      <c r="R19" s="67" t="n"/>
+      <c r="S19" s="68" t="n"/>
+      <c r="T19" s="102" t="inlineStr">
+        <is>
+          <t>OJK Compliance</t>
+        </is>
+      </c>
+      <c r="U19" s="112" t="inlineStr">
+        <is>
+          <t>Medium △</t>
+        </is>
+      </c>
+      <c r="V19" s="104" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1">
+      <c r="A20" s="105" t="n"/>
+      <c r="B20" s="106" t="n"/>
+      <c r="C20" s="108" t="n"/>
+      <c r="D20" s="108" t="n"/>
+      <c r="E20" s="108" t="n"/>
+      <c r="F20" s="108" t="n"/>
+      <c r="G20" s="108" t="n"/>
+      <c r="H20" s="108" t="n"/>
+      <c r="I20" s="108" t="n"/>
+      <c r="J20" s="108" t="n"/>
+      <c r="K20" s="108" t="n"/>
+      <c r="L20" s="108" t="n"/>
+      <c r="M20" s="108" t="n"/>
+      <c r="N20" s="108" t="n"/>
+      <c r="O20" s="108" t="n"/>
+      <c r="P20" s="108" t="n"/>
+      <c r="Q20" s="108" t="n"/>
+      <c r="R20" s="108" t="n"/>
+      <c r="S20" s="108" t="n"/>
+      <c r="T20" s="109" t="inlineStr"/>
+      <c r="U20" s="109" t="inlineStr"/>
+      <c r="V20" s="109" t="inlineStr"/>
+    </row>
+    <row r="21" ht="14" customHeight="1"/>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="115" t="inlineStr">
+        <is>
+          <t>REVENUE LINKAGE</t>
+        </is>
+      </c>
+      <c r="T22" s="90" t="inlineStr">
+        <is>
+          <t>REVENUE DASHBOARD</t>
+        </is>
+      </c>
+      <c r="U22" s="67" t="n"/>
+      <c r="V22" s="68" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="91" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B23" s="67" t="n"/>
+      <c r="C23" s="67" t="n"/>
+      <c r="D23" s="67" t="n"/>
+      <c r="E23" s="67" t="n"/>
+      <c r="F23" s="67" t="n"/>
+      <c r="G23" s="68" t="n"/>
+      <c r="H23" s="91" t="inlineStr">
+        <is>
+          <t>Revenue Unlock</t>
+        </is>
+      </c>
+      <c r="I23" s="67" t="n"/>
+      <c r="J23" s="67" t="n"/>
+      <c r="K23" s="67" t="n"/>
+      <c r="L23" s="67" t="n"/>
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="91" t="inlineStr">
+        <is>
+          <t>Est. Monthly Value</t>
+        </is>
+      </c>
+      <c r="O23" s="67" t="n"/>
+      <c r="P23" s="67" t="n"/>
+      <c r="Q23" s="68" t="n"/>
+      <c r="R23" s="91" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="S23" s="68" t="n"/>
+      <c r="T23" s="95" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="U23" s="95" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="V23" s="95" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="116" t="inlineStr">
+        <is>
+          <t>Platform Prototype Live</t>
+        </is>
+      </c>
+      <c r="B24" s="67" t="n"/>
+      <c r="C24" s="67" t="n"/>
+      <c r="D24" s="67" t="n"/>
+      <c r="E24" s="67" t="n"/>
+      <c r="F24" s="67" t="n"/>
+      <c r="G24" s="68" t="n"/>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="49" t="n"/>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="49" t="n"/>
+      <c r="L24" s="49" t="n"/>
+      <c r="M24" s="49" t="n"/>
+      <c r="N24" s="117" t="inlineStr">
+        <is>
+          <t>Rp —</t>
+        </is>
+      </c>
+      <c r="O24" s="67" t="n"/>
+      <c r="P24" s="67" t="n"/>
+      <c r="Q24" s="68" t="n"/>
+      <c r="R24" s="88" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="S24" s="68" t="n"/>
+      <c r="T24" s="102" t="inlineStr">
+        <is>
+          <t>Enables Partners</t>
+        </is>
+      </c>
+      <c r="U24" s="104" t="inlineStr">
+        <is>
+          <t>Rp —</t>
+        </is>
+      </c>
+      <c r="V24" s="112" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="118" t="inlineStr">
+        <is>
+          <t>Backend APIs Live</t>
+        </is>
+      </c>
+      <c r="B25" s="67" t="n"/>
+      <c r="C25" s="67" t="n"/>
+      <c r="D25" s="67" t="n"/>
+      <c r="E25" s="67" t="n"/>
+      <c r="F25" s="67" t="n"/>
+      <c r="G25" s="68" t="n"/>
+      <c r="H25" s="119" t="n"/>
+      <c r="I25" s="119" t="n"/>
+      <c r="J25" s="119" t="n"/>
+      <c r="K25" s="119" t="n"/>
+      <c r="L25" s="119" t="n"/>
+      <c r="M25" s="119" t="n"/>
+      <c r="N25" s="120" t="inlineStr">
+        <is>
+          <t>Rp 50jt / mo</t>
+        </is>
+      </c>
+      <c r="O25" s="67" t="n"/>
+      <c r="P25" s="67" t="n"/>
+      <c r="Q25" s="68" t="n"/>
+      <c r="R25" s="88" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="S25" s="68" t="n"/>
+      <c r="T25" s="121" t="inlineStr">
+        <is>
+          <t>Pilot Revenue</t>
+        </is>
+      </c>
+      <c r="U25" s="122" t="inlineStr">
+        <is>
+          <t>Rp 50jt / mo</t>
+        </is>
+      </c>
+      <c r="V25" s="112" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="116" t="inlineStr">
+        <is>
+          <t>1,000 Merchants Onboarded</t>
+        </is>
+      </c>
+      <c r="B26" s="67" t="n"/>
+      <c r="C26" s="67" t="n"/>
+      <c r="D26" s="67" t="n"/>
+      <c r="E26" s="67" t="n"/>
+      <c r="F26" s="67" t="n"/>
+      <c r="G26" s="68" t="n"/>
+      <c r="H26" s="123" t="n"/>
+      <c r="I26" s="123" t="n"/>
+      <c r="J26" s="123" t="n"/>
+      <c r="K26" s="123" t="n"/>
+      <c r="L26" s="123" t="n"/>
+      <c r="M26" s="123" t="n"/>
+      <c r="N26" s="117" t="inlineStr">
+        <is>
+          <t>Rp 500jt / mo</t>
+        </is>
+      </c>
+      <c r="O26" s="67" t="n"/>
+      <c r="P26" s="67" t="n"/>
+      <c r="Q26" s="68" t="n"/>
+      <c r="R26" s="89" t="inlineStr">
+        <is>
+          <t>At Risk</t>
+        </is>
+      </c>
+      <c r="S26" s="68" t="n"/>
+      <c r="T26" s="102" t="inlineStr">
+        <is>
+          <t>Full Monetization</t>
+        </is>
+      </c>
+      <c r="U26" s="104" t="inlineStr">
+        <is>
+          <t>Rp 500jt / mo</t>
+        </is>
+      </c>
+      <c r="V26" s="103" t="inlineStr">
+        <is>
+          <t>At Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="124" t="inlineStr">
+        <is>
+          <t>Confidential — Internal Program Governance  |  Olsera Mitra Modal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="64">
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="O7:V7"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="O10:V10"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="O6:V6"/>
+    <mergeCell ref="A22:S22"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="N24:Q24"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="A17:B18"/>
+    <mergeCell ref="A4:V4"/>
+    <mergeCell ref="P15:S15"/>
+    <mergeCell ref="O9:V9"/>
+    <mergeCell ref="H7:M7"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="A28:V28"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="N26:Q26"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="A19:B20"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="O5:V5"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="N25:Q25"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="H5:M5"/>
+    <mergeCell ref="A15:B16"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="H23:M23"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="H8:M8"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="L14:O14"/>
+    <mergeCell ref="N23:Q23"/>
+    <mergeCell ref="O8:V8"/>
+    <mergeCell ref="H10:M10"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H9:M9"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="A12:V12"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="0.5" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="125" t="inlineStr">
+        <is>
+          <t>OLSERA MITRA MODAL — PROGRAM MASTER TIMELINE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="126" t="inlineStr">
+        <is>
+          <t>Financial Infrastructure Development &amp; Commercial Rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="127" t="inlineStr">
+        <is>
+          <t>Executive Summary</t>
+        </is>
+      </c>
+      <c r="N4" s="127" t="inlineStr">
+        <is>
+          <t>Dependencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="91" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B5" s="91" t="inlineStr">
+        <is>
+          <t>Objective</t>
+        </is>
+      </c>
+      <c r="C5" s="91" t="inlineStr">
+        <is>
+          <t>Key Deliverable</t>
+        </is>
+      </c>
+      <c r="D5" s="91" t="inlineStr">
+        <is>
+          <t>Target Go Live</t>
+        </is>
+      </c>
+      <c r="E5" s="91" t="inlineStr">
+        <is>
+          <t>Revenue Impact</t>
+        </is>
+      </c>
+      <c r="F5" s="91" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="G5" s="91" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="N5" s="90" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="O5" s="90" t="inlineStr">
+        <is>
+          <t>Depends On</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="128" t="inlineStr">
+        <is>
+          <t>Phase 1 — Foundation</t>
+        </is>
+      </c>
+      <c r="B6" s="129" t="inlineStr">
+        <is>
+          <t>Core Platform Build</t>
+        </is>
+      </c>
+      <c r="C6" s="130" t="inlineStr">
+        <is>
+          <t>5-portal prototype live</t>
+        </is>
+      </c>
+      <c r="D6" s="131" t="inlineStr">
+        <is>
+          <t>30 Apr 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="130" t="inlineStr">
+        <is>
+          <t>Enables Partner Onboarding</t>
+        </is>
+      </c>
+      <c r="F6" s="88" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G6" s="132" t="inlineStr">
+        <is>
+          <t>Product / Engineering</t>
+        </is>
+      </c>
+      <c r="N6" s="116" t="inlineStr">
+        <is>
+          <t>Partner API Access</t>
+        </is>
+      </c>
+      <c r="O6" s="130" t="inlineStr">
+        <is>
+          <t>External Parties (Adapundi, OCBC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="133" t="inlineStr">
+        <is>
+          <t>Phase 2 — Integration</t>
+        </is>
+      </c>
+      <c r="B7" s="134" t="inlineStr">
+        <is>
+          <t>Bank &amp; Partner API Integration</t>
+        </is>
+      </c>
+      <c r="C7" s="135" t="inlineStr">
+        <is>
+          <t>Backend APIs + Partner MOU</t>
+        </is>
+      </c>
+      <c r="D7" s="136" t="inlineStr">
+        <is>
+          <t>17 May 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="135" t="inlineStr">
+        <is>
+          <t>Pilot Revenue Start</t>
+        </is>
+      </c>
+      <c r="F7" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G7" s="137" t="inlineStr">
+        <is>
+          <t>Product / Engineering</t>
+        </is>
+      </c>
+      <c r="N7" s="118" t="inlineStr">
+        <is>
+          <t>Data Schema Final.</t>
+        </is>
+      </c>
+      <c r="O7" s="135" t="inlineStr">
+        <is>
+          <t>Core Build / E9 DB Migrations</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="128" t="inlineStr">
+        <is>
+          <t>Phase 3 — Commercialization</t>
+        </is>
+      </c>
+      <c r="B8" s="129" t="inlineStr">
+        <is>
+          <t>Merchant Rollout</t>
+        </is>
+      </c>
+      <c r="C8" s="130" t="inlineStr">
+        <is>
+          <t>1,000 Merchants Onboarded</t>
+        </is>
+      </c>
+      <c r="D8" s="131" t="inlineStr">
+        <is>
+          <t>30 Jul 2026</t>
+        </is>
+      </c>
+      <c r="E8" s="130" t="inlineStr">
+        <is>
+          <t>Monetization Start</t>
+        </is>
+      </c>
+      <c r="F8" s="89" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G8" s="132" t="inlineStr">
+        <is>
+          <t>Product / Engineering</t>
+        </is>
+      </c>
+      <c r="N8" s="116" t="inlineStr">
+        <is>
+          <t>OJK Compliance</t>
+        </is>
+      </c>
+      <c r="O8" s="130" t="inlineStr">
+        <is>
+          <t>Scoring Engine / Legal Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="12" customHeight="1"/>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="127" t="inlineStr">
+        <is>
+          <t>Module Timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="91" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B11" s="91" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="C11" s="91" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D11" s="91" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="E11" s="91" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="F11" s="91" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="G11" s="91" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H11" s="91" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="I11" s="91" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="J11" s="91" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="K11" s="91" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="L11" s="91" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="N11" s="90" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="O11" s="90" t="inlineStr">
+        <is>
+          <t>Impact If Late</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="128" t="inlineStr">
+        <is>
+          <t>Merchant Flow Engine</t>
+        </is>
+      </c>
+      <c r="B12" s="129" t="inlineStr">
+        <is>
+          <t>Core Platform Build</t>
+        </is>
+      </c>
+      <c r="C12" s="132" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D12" s="132" t="inlineStr">
+        <is>
+          <t>01-Mar-26</t>
+        </is>
+      </c>
+      <c r="E12" s="132" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="F12" s="138" t="inlineStr">
+        <is>
+          <t>E1, E2 Foundation</t>
+        </is>
+      </c>
+      <c r="G12" s="87" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="H12" s="139" t="n"/>
+      <c r="I12" s="140" t="n"/>
+      <c r="J12" s="140" t="n"/>
+      <c r="K12" s="140" t="n"/>
+      <c r="L12" s="140" t="n"/>
+      <c r="N12" s="102" t="inlineStr">
+        <is>
+          <t>Merchant Prototype</t>
+        </is>
+      </c>
+      <c r="O12" s="138" t="inlineStr">
+        <is>
+          <t>On track — no blockers</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="133" t="inlineStr">
+        <is>
+          <t>Scoring Engine</t>
+        </is>
+      </c>
+      <c r="B13" s="134" t="inlineStr">
+        <is>
+          <t>Scoring Model Ready</t>
+        </is>
+      </c>
+      <c r="C13" s="137" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D13" s="137" t="inlineStr">
+        <is>
+          <t>10-Mar-26</t>
+        </is>
+      </c>
+      <c r="E13" s="137" t="inlineStr">
+        <is>
+          <t>20-Mar-26</t>
+        </is>
+      </c>
+      <c r="F13" s="141" t="inlineStr">
+        <is>
+          <t>E1 DB Schema</t>
+        </is>
+      </c>
+      <c r="G13" s="88" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H13" s="142" t="n"/>
+      <c r="I13" s="143" t="n"/>
+      <c r="J13" s="143" t="n"/>
+      <c r="K13" s="143" t="n"/>
+      <c r="L13" s="143" t="n"/>
+      <c r="N13" s="121" t="inlineStr">
+        <is>
+          <t>Scoring Engine</t>
+        </is>
+      </c>
+      <c r="O13" s="141" t="inlineStr">
+        <is>
+          <t>Delays push merchant API</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="128" t="inlineStr">
+        <is>
+          <t>Partner Portal</t>
+        </is>
+      </c>
+      <c r="B14" s="129" t="inlineStr">
+        <is>
+          <t>Partner Decision Flow</t>
+        </is>
+      </c>
+      <c r="C14" s="132" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D14" s="132" t="inlineStr">
+        <is>
+          <t>01-Apr-26</t>
+        </is>
+      </c>
+      <c r="E14" s="132" t="inlineStr">
+        <is>
+          <t>15-Apr-26</t>
+        </is>
+      </c>
+      <c r="F14" s="138" t="inlineStr">
+        <is>
+          <t>E4 + Partner MOU ⚠</t>
+        </is>
+      </c>
+      <c r="G14" s="89" t="inlineStr">
+        <is>
+          <t>At Risk</t>
+        </is>
+      </c>
+      <c r="H14" s="140" t="n"/>
+      <c r="I14" s="144" t="n"/>
+      <c r="J14" s="140" t="n"/>
+      <c r="K14" s="140" t="n"/>
+      <c r="L14" s="140" t="n"/>
+      <c r="N14" s="102" t="inlineStr">
+        <is>
+          <t>Partner MOU</t>
+        </is>
+      </c>
+      <c r="O14" s="138" t="inlineStr">
+        <is>
+          <t>Portal unusable without partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="133" t="inlineStr">
+        <is>
+          <t>Admin &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B15" s="134" t="inlineStr">
+        <is>
+          <t>Operations Layer</t>
+        </is>
+      </c>
+      <c r="C15" s="137" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="137" t="inlineStr">
+        <is>
+          <t>15-Apr-26</t>
+        </is>
+      </c>
+      <c r="E15" s="137" t="inlineStr">
+        <is>
+          <t>30-Apr-26</t>
+        </is>
+      </c>
+      <c r="F15" s="141" t="inlineStr">
+        <is>
+          <t>E5 Partner Portal</t>
+        </is>
+      </c>
+      <c r="G15" s="87" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="H15" s="143" t="n"/>
+      <c r="I15" s="145" t="n"/>
+      <c r="J15" s="143" t="n"/>
+      <c r="K15" s="143" t="n"/>
+      <c r="L15" s="143" t="n"/>
+      <c r="N15" s="121" t="inlineStr">
+        <is>
+          <t>Partner Portal</t>
+        </is>
+      </c>
+      <c r="O15" s="141" t="inlineStr">
+        <is>
+          <t>Admin blind without data</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="128" t="inlineStr">
+        <is>
+          <t>Backend APIs</t>
+        </is>
+      </c>
+      <c r="B16" s="129" t="inlineStr">
+        <is>
+          <t>Full API Integration</t>
+        </is>
+      </c>
+      <c r="C16" s="132" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D16" s="132" t="inlineStr">
+        <is>
+          <t>01-May-26</t>
+        </is>
+      </c>
+      <c r="E16" s="132" t="inlineStr">
+        <is>
+          <t>31-May-26</t>
+        </is>
+      </c>
+      <c r="F16" s="138" t="inlineStr">
+        <is>
+          <t>E9 DB + E7 Scoring</t>
+        </is>
+      </c>
+      <c r="G16" s="114" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="H16" s="140" t="n"/>
+      <c r="I16" s="140" t="n"/>
+      <c r="J16" s="146" t="n"/>
+      <c r="K16" s="140" t="n"/>
+      <c r="L16" s="140" t="n"/>
+      <c r="N16" s="102" t="inlineStr">
+        <is>
+          <t>DB Migrations</t>
+        </is>
+      </c>
+      <c r="O16" s="138" t="inlineStr">
+        <is>
+          <t>All APIs blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="133" t="inlineStr">
+        <is>
+          <t>Partner API Integ.</t>
+        </is>
+      </c>
+      <c r="B17" s="134" t="inlineStr">
+        <is>
+          <t>Adapundi + OCBC Full API</t>
+        </is>
+      </c>
+      <c r="C17" s="137" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="D17" s="137" t="inlineStr">
+        <is>
+          <t>01-Jun-26</t>
+        </is>
+      </c>
+      <c r="E17" s="137" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="F17" s="141" t="inlineStr">
+        <is>
+          <t>API docs from partners ⚠</t>
+        </is>
+      </c>
+      <c r="G17" s="89" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="H17" s="143" t="n"/>
+      <c r="I17" s="143" t="n"/>
+      <c r="J17" s="143" t="n"/>
+      <c r="K17" s="147" t="n"/>
+      <c r="L17" s="143" t="n"/>
+      <c r="N17" s="121" t="inlineStr">
+        <is>
+          <t>Partner API Docs</t>
+        </is>
+      </c>
+      <c r="O17" s="141" t="inlineStr">
+        <is>
+          <t>Integration cannot start</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="12" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="127" t="inlineStr">
+        <is>
+          <t>Revenue Linkage</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="91" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B20" s="91" t="inlineStr">
+        <is>
+          <t>Revenue Unlock</t>
+        </is>
+      </c>
+      <c r="C20" s="91" t="inlineStr">
+        <is>
+          <t>Est Monthly Value</t>
+        </is>
+      </c>
+      <c r="D20" s="91" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="116" t="inlineStr">
+        <is>
+          <t>Platform Prototype Live</t>
+        </is>
+      </c>
+      <c r="B21" s="129" t="inlineStr">
+        <is>
+          <t>Enables Partner Onboarding</t>
+        </is>
+      </c>
+      <c r="C21" s="117" t="inlineStr">
+        <is>
+          <t>Rp —</t>
+        </is>
+      </c>
+      <c r="D21" s="87" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>Backend APIs Live</t>
+        </is>
+      </c>
+      <c r="B22" s="134" t="inlineStr">
+        <is>
+          <t>Pilot Revenue Start</t>
+        </is>
+      </c>
+      <c r="C22" s="120" t="inlineStr">
+        <is>
+          <t>Rp 50jt / mo</t>
+        </is>
+      </c>
+      <c r="D22" s="88" t="inlineStr">
+        <is>
+          <t>YELLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="116" t="inlineStr">
+        <is>
+          <t>1,000 Merchants Onboard</t>
+        </is>
+      </c>
+      <c r="B23" s="129" t="inlineStr">
+        <is>
+          <t>Full Monetization</t>
+        </is>
+      </c>
+      <c r="C23" s="117" t="inlineStr">
+        <is>
+          <t>Rp 500jt / mo</t>
+        </is>
+      </c>
+      <c r="D23" s="89" t="inlineStr">
+        <is>
+          <t>At Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="124" t="inlineStr">
+        <is>
+          <t>Internal — Program Governance Use Only  |  Olsera Mitra Modal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A25:O25"/>
+    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="N4:O4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(roadmap): update timeline per meeting feedback
New delivery schedule:
- Backoffice Adapundi: akhir Maret (unchanged)
- Backoffice OCBC: akhir April (was akhir Maret)
- Web Merchant (E4 + E12 Ph.1 redirect): akhir April (was 31 Mar)
- Web Partner portal (E5, E8): akhir Mei (was 15 Apr)
- Web Admin & Management (E6, E10): akhir Mei (was 30 Apr)

Updated across all 4 Excel sheets (deadlines, Gantt bars, module
end dates) and ROADMAP.md (phase table, epic tables, ASCII Gantt,
backoffice notes).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OMM-2026-Roadmap.xlsx
+++ b/docs/OMM-2026-Roadmap.xlsx
@@ -623,7 +623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="148">
+  <cellXfs count="151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1008,6 +1008,9 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1507,7 +1510,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>31 Mar</t>
+          <t>30 Apr</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1544,7 +1547,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>15 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1581,7 +1584,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>30 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1677,7 +1680,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>⚠️  Note — Backoffice version: A separate backoffice application (not this web app) also targets Adapundi + OCBC integration by end of March 2026.</t>
+          <t>⚠️  Note — Backoffice version: A separate backoffice application (not this web app) targets Adapundi integration by end of March 2026, and OCBC integration by end of April 2026.</t>
         </is>
       </c>
       <c r="B11" s="14" t="n"/>
@@ -1941,7 +1944,7 @@
       </c>
       <c r="C21" s="24" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1–Q2</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
@@ -1951,7 +1954,7 @@
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>31 Mar</t>
+          <t>30 Apr</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1984,7 +1987,7 @@
       </c>
       <c r="C22" s="24" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1–Q2</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
@@ -1994,7 +1997,7 @@
       </c>
       <c r="E22" s="24" t="inlineStr">
         <is>
-          <t>31 Mar</t>
+          <t>30 Apr</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -2016,7 +2019,7 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>E12 Phase 1: Adapundi redirect + OCBC 'Coming Soon' card — already live in prototype. Production deployment targets end of March. No API integration required.</t>
+          <t>E12 Phase 1: Adapundi redirect + OCBC 'Coming Soon' card — already live in prototype. Production deployment for web app targets end of April. No API integration required.</t>
         </is>
       </c>
       <c r="B23" s="14" t="n"/>
@@ -2064,7 +2067,7 @@
       </c>
       <c r="E25" s="24" t="inlineStr">
         <is>
-          <t>15 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
@@ -2106,7 +2109,7 @@
       </c>
       <c r="E26" s="28" t="inlineStr">
         <is>
-          <t>15 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
@@ -2148,7 +2151,7 @@
       </c>
       <c r="E27" s="28" t="inlineStr">
         <is>
-          <t>30 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
@@ -2190,7 +2193,7 @@
       </c>
       <c r="E28" s="28" t="inlineStr">
         <is>
-          <t>30 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -2853,7 +2856,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1–Q2</t>
         </is>
       </c>
       <c r="D9" s="61" t="inlineStr">
@@ -2868,17 +2871,17 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>31 Mar</t>
+          <t>30 Apr</t>
         </is>
       </c>
       <c r="G9" s="49" t="n"/>
       <c r="H9" s="49" t="n"/>
       <c r="I9" s="49" t="n"/>
       <c r="J9" s="49" t="n"/>
-      <c r="K9" s="45" t="n"/>
-      <c r="L9" s="45" t="n"/>
-      <c r="M9" s="45" t="n"/>
-      <c r="N9" s="45" t="n"/>
+      <c r="K9" s="49" t="n"/>
+      <c r="L9" s="49" t="n"/>
+      <c r="M9" s="49" t="n"/>
+      <c r="N9" s="49" t="n"/>
       <c r="O9" s="45" t="n"/>
       <c r="P9" s="45" t="n"/>
       <c r="Q9" s="45" t="n"/>
@@ -2901,7 +2904,7 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1–Q2</t>
         </is>
       </c>
       <c r="D10" s="50" t="inlineStr">
@@ -2916,17 +2919,17 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>31 Mar</t>
+          <t>30 Apr</t>
         </is>
       </c>
       <c r="G10" s="47" t="n"/>
       <c r="H10" s="47" t="n"/>
       <c r="I10" s="49" t="n"/>
       <c r="J10" s="49" t="n"/>
-      <c r="K10" s="47" t="n"/>
-      <c r="L10" s="47" t="n"/>
-      <c r="M10" s="47" t="n"/>
-      <c r="N10" s="47" t="n"/>
+      <c r="K10" s="49" t="n"/>
+      <c r="L10" s="49" t="n"/>
+      <c r="M10" s="49" t="n"/>
+      <c r="N10" s="49" t="n"/>
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="47" t="n"/>
       <c r="Q10" s="47" t="n"/>
@@ -2964,7 +2967,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>15 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="G11" s="45" t="n"/>
@@ -2973,12 +2976,12 @@
       <c r="J11" s="52" t="n"/>
       <c r="K11" s="52" t="n"/>
       <c r="L11" s="52" t="n"/>
-      <c r="M11" s="45" t="n"/>
-      <c r="N11" s="45" t="n"/>
-      <c r="O11" s="45" t="n"/>
-      <c r="P11" s="45" t="n"/>
-      <c r="Q11" s="45" t="n"/>
-      <c r="R11" s="45" t="n"/>
+      <c r="M11" s="52" t="n"/>
+      <c r="N11" s="52" t="n"/>
+      <c r="O11" s="52" t="n"/>
+      <c r="P11" s="52" t="n"/>
+      <c r="Q11" s="52" t="n"/>
+      <c r="R11" s="52" t="n"/>
       <c r="S11" s="45" t="n"/>
       <c r="T11" s="45" t="n"/>
       <c r="U11" s="45" t="n"/>
@@ -3012,7 +3015,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>15 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="G12" s="47" t="n"/>
@@ -3021,12 +3024,12 @@
       <c r="J12" s="52" t="n"/>
       <c r="K12" s="52" t="n"/>
       <c r="L12" s="52" t="n"/>
-      <c r="M12" s="47" t="n"/>
-      <c r="N12" s="47" t="n"/>
-      <c r="O12" s="47" t="n"/>
-      <c r="P12" s="47" t="n"/>
-      <c r="Q12" s="47" t="n"/>
-      <c r="R12" s="47" t="n"/>
+      <c r="M12" s="52" t="n"/>
+      <c r="N12" s="52" t="n"/>
+      <c r="O12" s="52" t="n"/>
+      <c r="P12" s="52" t="n"/>
+      <c r="Q12" s="52" t="n"/>
+      <c r="R12" s="52" t="n"/>
       <c r="S12" s="47" t="n"/>
       <c r="T12" s="47" t="n"/>
       <c r="U12" s="47" t="n"/>
@@ -3060,7 +3063,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>30 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="G13" s="45" t="n"/>
@@ -3071,10 +3074,10 @@
       <c r="L13" s="52" t="n"/>
       <c r="M13" s="52" t="n"/>
       <c r="N13" s="52" t="n"/>
-      <c r="O13" s="45" t="n"/>
-      <c r="P13" s="45" t="n"/>
-      <c r="Q13" s="45" t="n"/>
-      <c r="R13" s="45" t="n"/>
+      <c r="O13" s="52" t="n"/>
+      <c r="P13" s="52" t="n"/>
+      <c r="Q13" s="52" t="n"/>
+      <c r="R13" s="52" t="n"/>
       <c r="S13" s="45" t="n"/>
       <c r="T13" s="45" t="n"/>
       <c r="U13" s="45" t="n"/>
@@ -3108,7 +3111,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>30 Apr</t>
+          <t>31 May</t>
         </is>
       </c>
       <c r="G14" s="47" t="n"/>
@@ -3119,10 +3122,10 @@
       <c r="L14" s="52" t="n"/>
       <c r="M14" s="52" t="n"/>
       <c r="N14" s="52" t="n"/>
-      <c r="O14" s="47" t="n"/>
-      <c r="P14" s="47" t="n"/>
-      <c r="Q14" s="47" t="n"/>
-      <c r="R14" s="47" t="n"/>
+      <c r="O14" s="52" t="n"/>
+      <c r="P14" s="52" t="n"/>
+      <c r="Q14" s="52" t="n"/>
+      <c r="R14" s="52" t="n"/>
       <c r="S14" s="47" t="n"/>
       <c r="T14" s="47" t="n"/>
       <c r="U14" s="47" t="n"/>
@@ -3562,7 +3565,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="78" t="inlineStr">
         <is>
-          <t>Core Platform Build</t>
+          <t>Core Platform Build + Web Merchant Flow</t>
         </is>
       </c>
       <c r="B7" s="67" t="n"/>
@@ -3577,7 +3580,7 @@
       </c>
       <c r="H7" s="79" t="inlineStr">
         <is>
-          <t>Backend APIs &amp; Partner Portal</t>
+          <t>Backend APIs + Partner &amp; Admin Portals</t>
         </is>
       </c>
       <c r="I7" s="67" t="n"/>
@@ -3606,7 +3609,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="81" t="inlineStr">
         <is>
-          <t>5-portal prototype • Auth • Scoring engine</t>
+          <t>5-portal prototype • Auth • Scoring engine • Merchant web (Apr)</t>
         </is>
       </c>
       <c r="B8" s="67" t="n"/>
@@ -3617,7 +3620,7 @@
       <c r="G8" s="72" t="inlineStr"/>
       <c r="H8" s="82" t="inlineStr">
         <is>
-          <t>All API endpoints live • Partner MOU required</t>
+          <t>All API endpoints live • Partner MOU required • Admin &amp; Mgmt (May)</t>
         </is>
       </c>
       <c r="I8" s="67" t="n"/>
@@ -3992,7 +3995,7 @@
         <is>
           <t>System Testing
 &amp; QA
-(May)</t>
+(May – Jun)</t>
         </is>
       </c>
       <c r="B19" s="101" t="n"/>
@@ -4523,7 +4526,7 @@
       </c>
       <c r="D7" s="136" t="inlineStr">
         <is>
-          <t>17 May 2026</t>
+          <t>31 May 2026</t>
         </is>
       </c>
       <c r="E7" s="135" t="inlineStr">
@@ -4702,7 +4705,7 @@
       </c>
       <c r="E12" s="132" t="inlineStr">
         <is>
-          <t>31-Mar-26</t>
+          <t>30-Apr-26</t>
         </is>
       </c>
       <c r="F12" s="138" t="inlineStr">
@@ -4716,7 +4719,7 @@
         </is>
       </c>
       <c r="H12" s="139" t="n"/>
-      <c r="I12" s="140" t="n"/>
+      <c r="I12" s="148" t="n"/>
       <c r="J12" s="140" t="n"/>
       <c r="K12" s="140" t="n"/>
       <c r="L12" s="140" t="n"/>
@@ -4806,7 +4809,7 @@
       </c>
       <c r="E14" s="132" t="inlineStr">
         <is>
-          <t>15-Apr-26</t>
+          <t>31-May-26</t>
         </is>
       </c>
       <c r="F14" s="138" t="inlineStr">
@@ -4821,7 +4824,7 @@
       </c>
       <c r="H14" s="140" t="n"/>
       <c r="I14" s="144" t="n"/>
-      <c r="J14" s="140" t="n"/>
+      <c r="J14" s="149" t="n"/>
       <c r="K14" s="140" t="n"/>
       <c r="L14" s="140" t="n"/>
       <c r="N14" s="102" t="inlineStr">
@@ -4858,7 +4861,7 @@
       </c>
       <c r="E15" s="137" t="inlineStr">
         <is>
-          <t>30-Apr-26</t>
+          <t>31-May-26</t>
         </is>
       </c>
       <c r="F15" s="141" t="inlineStr">
@@ -4873,7 +4876,7 @@
       </c>
       <c r="H15" s="143" t="n"/>
       <c r="I15" s="145" t="n"/>
-      <c r="J15" s="143" t="n"/>
+      <c r="J15" s="150" t="n"/>
       <c r="K15" s="143" t="n"/>
       <c r="L15" s="143" t="n"/>
       <c r="N15" s="121" t="inlineStr">

</xml_diff>